<commit_message>
new versions of French and English CVs
</commit_message>
<xml_diff>
--- a/Data/ArthurHeimCareerDataEn.xlsx
+++ b/Data/ArthurHeimCareerDataEn.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arthurheim/Library/CloudStorage/Dropbox/Travail_encrypted_decrypted/PHD/career/Data_DrivenResume/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455CBB3B-12C5-4E4E-B056-CCBC8579AC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110C1282-D94F-8C45-B276-F82D24E2986A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8220" yWindow="500" windowWidth="27240" windowHeight="19200" activeTab="10" xr2:uid="{65AA7443-0872-B84D-B38F-A133D7C4ED29}"/>
+    <workbookView xWindow="8220" yWindow="500" windowWidth="27240" windowHeight="19200" activeTab="9" xr2:uid="{65AA7443-0872-B84D-B38F-A133D7C4ED29}"/>
   </bookViews>
   <sheets>
     <sheet name="education" sheetId="1" r:id="rId1"/>
@@ -694,9 +694,6 @@
     <t>Completed</t>
   </si>
   <si>
-    <t>POSAJE: Multi-arm RCT to foster access to formal early childcare</t>
-  </si>
-  <si>
     <t>ISAJE: Market design experiment of daycare assignments with random tie-breaks</t>
   </si>
   <si>
@@ -977,6 +974,9 @@
   </si>
   <si>
     <t>Conférence | Numérique en commun[s] 2025</t>
+  </si>
+  <si>
+    <t>Baby steps: Multi-arm RCT to foster access to formal early childcare</t>
   </si>
 </sst>
 </file>
@@ -1535,13 +1535,13 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D2" t="s">
         <v>57</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="34">
@@ -1626,7 +1626,7 @@
         <v>19</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -1634,16 +1634,16 @@
         <v>203</v>
       </c>
       <c r="B2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C2" t="s">
         <v>193</v>
       </c>
       <c r="D2" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="E2" s="26" t="s">
         <v>233</v>
-      </c>
-      <c r="E2" s="26" t="s">
-        <v>234</v>
       </c>
       <c r="F2" t="s">
         <v>198</v>
@@ -1652,24 +1652,24 @@
         <v>205</v>
       </c>
       <c r="H2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>206</v>
+        <v>288</v>
       </c>
       <c r="B3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C3" t="s">
         <v>194</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F3" t="s">
         <v>197</v>
@@ -1678,24 +1678,24 @@
         <v>205</v>
       </c>
       <c r="H3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C4" t="s">
         <v>195</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E4" s="26" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F4" t="s">
         <v>199</v>
@@ -1704,24 +1704,24 @@
         <v>205</v>
       </c>
       <c r="H4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C5" t="s">
         <v>195</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F5" t="s">
         <v>200</v>
@@ -1730,50 +1730,50 @@
         <v>204</v>
       </c>
       <c r="H5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C6" t="s">
         <v>196</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G6" t="s">
         <v>204</v>
       </c>
       <c r="H6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
+        <v>208</v>
+      </c>
+      <c r="B7" t="s">
         <v>209</v>
-      </c>
-      <c r="B7" t="s">
-        <v>210</v>
       </c>
       <c r="C7" t="s">
         <v>196</v>
       </c>
       <c r="D7" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="E7" s="26" t="s">
         <v>235</v>
-      </c>
-      <c r="E7" s="26" t="s">
-        <v>236</v>
       </c>
       <c r="F7" t="s">
         <v>201</v>
@@ -1782,18 +1782,18 @@
         <v>204</v>
       </c>
       <c r="H7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B8" t="s">
         <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D8">
         <v>2013</v>
@@ -1802,18 +1802,18 @@
         <v>2014</v>
       </c>
       <c r="F8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G8" t="s">
         <v>205</v>
       </c>
       <c r="H8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B9" t="s">
         <v>39</v>
@@ -1828,13 +1828,13 @@
         <v>2016</v>
       </c>
       <c r="F9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G9" t="s">
         <v>205</v>
       </c>
       <c r="H9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -1874,16 +1874,16 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>286</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>287</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4" t="s">
@@ -1893,16 +1893,16 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B3" t="s">
+        <v>253</v>
+      </c>
+      <c r="C3" t="s">
         <v>254</v>
       </c>
-      <c r="C3" t="s">
-        <v>255</v>
-      </c>
       <c r="D3" s="28" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F3" t="s">
         <v>21</v>
@@ -1937,7 +1937,7 @@
         <v>103</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F5" t="s">
         <v>21</v>
@@ -1962,7 +1962,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
@@ -1979,7 +1979,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B8" t="s">
         <v>108</v>
@@ -1996,7 +1996,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B9" t="s">
         <v>106</v>
@@ -2013,7 +2013,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B10" t="s">
         <v>105</v>
@@ -2030,10 +2030,10 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
+        <v>263</v>
+      </c>
+      <c r="B11" t="s">
         <v>264</v>
-      </c>
-      <c r="B11" t="s">
-        <v>265</v>
       </c>
       <c r="C11" t="s">
         <v>103</v>
@@ -2047,7 +2047,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B12" t="s">
         <v>104</v>
@@ -2064,7 +2064,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B13" t="s">
         <v>102</v>
@@ -2153,7 +2153,7 @@
         <v>81</v>
       </c>
       <c r="G3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -2258,7 +2258,7 @@
         <v>20</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>21</v>
@@ -2413,10 +2413,10 @@
         <v>180</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D2" s="4">
         <v>2025</v>
@@ -2425,7 +2425,7 @@
         <v>148</v>
       </c>
       <c r="F2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>21</v>
@@ -2445,13 +2445,13 @@
         <v>177</v>
       </c>
       <c r="D3" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="E3" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="E3" s="12" t="s">
-        <v>230</v>
-      </c>
       <c r="F3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G3" t="s">
         <v>21</v>
@@ -2471,13 +2471,13 @@
         <v>102</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G4" t="s">
         <v>21</v>
@@ -2491,13 +2491,13 @@
         <v>180</v>
       </c>
       <c r="B5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C5" t="s">
         <v>103</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>148</v>
@@ -2517,16 +2517,16 @@
         <v>180</v>
       </c>
       <c r="B6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C6" t="s">
         <v>103</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F6" t="s">
         <v>182</v>
@@ -2600,7 +2600,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B3" t="s">
         <v>154</v>
@@ -2633,13 +2633,13 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B6" t="s">
         <v>157</v>
       </c>
       <c r="C6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2890,19 +2890,19 @@
     </row>
     <row r="2" spans="1:5" ht="119">
       <c r="A2" s="31" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B2" s="31">
         <v>2025</v>
       </c>
       <c r="C2" s="31" t="s">
+        <v>275</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>279</v>
+      </c>
+      <c r="E2" s="32" t="s">
         <v>276</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>280</v>
-      </c>
-      <c r="E2" s="32" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -3311,7 +3311,7 @@
         <v>67</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E6" s="23">
         <v>2024</v>
@@ -3381,7 +3381,7 @@
         <v>119</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E9" s="23">
         <v>2024</v>
@@ -3409,7 +3409,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="17">
       <c r="A1" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B1" s="20" t="s">
         <v>61</v>
@@ -3438,14 +3438,14 @@
     </row>
     <row r="2" spans="1:9" ht="136">
       <c r="A2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B2" s="23"/>
       <c r="C2" s="23" t="s">
         <v>51</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E2" s="23" t="s">
         <v>191</v>
@@ -3454,7 +3454,7 @@
         <v>2024</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H2" s="23" t="s">
         <v>21</v>
@@ -3465,11 +3465,11 @@
     </row>
     <row r="3" spans="1:9" ht="289">
       <c r="A3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B3" s="23"/>
       <c r="C3" s="23" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D3" s="23" t="s">
         <v>44</v>
@@ -3481,36 +3481,36 @@
         <v>2024</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H3" s="23" t="s">
         <v>21</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="119">
       <c r="A4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>60</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F4" s="23">
         <v>2024</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H4" s="23" t="s">
         <v>21</v>
@@ -3521,11 +3521,11 @@
     </row>
     <row r="5" spans="1:9" ht="306">
       <c r="A5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B5" s="23"/>
       <c r="C5" s="23" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D5" s="23" t="s">
         <v>50</v>
@@ -3537,7 +3537,7 @@
         <v>2024</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H5" s="23" t="s">
         <v>21</v>
@@ -3548,23 +3548,23 @@
     </row>
     <row r="6" spans="1:9" ht="153">
       <c r="A6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B6" s="23"/>
       <c r="C6" s="23" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D6" s="23" t="s">
         <v>67</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F6" s="23">
         <v>2025</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H6" s="23" t="s">
         <v>21</v>
@@ -3621,7 +3621,7 @@
     </row>
     <row r="9" spans="1:9" ht="68">
       <c r="A9" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B9" s="23"/>
       <c r="C9" s="25" t="s">
@@ -3631,13 +3631,13 @@
         <v>119</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F9" s="23">
         <v>2025</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H9" s="23" t="s">
         <v>21</v>

</xml_diff>